<commit_message>
Fix most active trades volume and turnover fields
</commit_message>
<xml_diff>
--- a/CSE_Stock_Trend_Analyzer.xlsx
+++ b/CSE_Stock_Trend_Analyzer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\CSE Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:20001_{A3F51F6A-6045-4492-9573-29D0B8ACB1B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A69FE4-574C-41B7-8E5A-0CDACB33FB72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="🇱🇰 CSE LIVE PRICES" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,6 @@
     <sheet name="📈 DASHBOARD" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,12 +38,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="317">
   <si>
     <t>🇱🇰   CSE LIVE PRICES  —  Colombo Stock Exchange</t>
   </si>
   <si>
-    <t>Last updated: 2026-05-29  13:41:50   |   Source: cse.lk   |   Currency: LKR</t>
+    <t>Last updated: 2026-05-29  14:17:39   |   Source: cse.lk   |   Currency: LKR</t>
   </si>
   <si>
     <t>Symbol</t>
@@ -74,7 +73,7 @@
     <t>COMMERCIAL BANK OF CEYLON PLC</t>
   </si>
   <si>
-    <t>2026-05-29 13:41</t>
+    <t>2026-05-29 14:17</t>
   </si>
   <si>
     <t>LOLC.N0000</t>
@@ -158,7 +157,13 @@
     <t>SMOT.N0000</t>
   </si>
   <si>
-    <t>SINH.N0000</t>
+    <t>MHDL.N0000</t>
+  </si>
+  <si>
+    <t>INME.N0000</t>
+  </si>
+  <si>
+    <t>LWL.N0000</t>
   </si>
   <si>
     <t>OFEQ.N0000</t>
@@ -176,43 +181,40 @@
     <t>UBF.N0000</t>
   </si>
   <si>
-    <t>CITH.N0000</t>
+    <t>KPHL.N0000</t>
   </si>
   <si>
     <t>UDPL.N0000</t>
   </si>
   <si>
+    <t>LALU.N0000</t>
+  </si>
+  <si>
+    <t>HNBF.N0000</t>
+  </si>
+  <si>
+    <t>TPL.N0000</t>
+  </si>
+  <si>
+    <t>ETWO.N0000</t>
+  </si>
+  <si>
     <t>SHOT.X0000</t>
   </si>
   <si>
-    <t>HNBF.N0000</t>
-  </si>
-  <si>
-    <t>CFVF.N0000</t>
-  </si>
-  <si>
-    <t>ETWO.N0000</t>
+    <t>SIL.N0000</t>
   </si>
   <si>
     <t>COMD.N0000</t>
   </si>
   <si>
-    <t>LGL.X0000</t>
-  </si>
-  <si>
-    <t>COCO.N0000</t>
-  </si>
-  <si>
-    <t>AUTO.N0000</t>
-  </si>
-  <si>
-    <t>KPHL.N0000</t>
-  </si>
-  <si>
     <t>🔥  MOST ACTIVE TRADES  (by Volume)</t>
   </si>
   <si>
-    <t>Volume</t>
+    <t>Turnover (LKR)</t>
+  </si>
+  <si>
+    <t>Share Volume</t>
   </si>
   <si>
     <t>CWL.N0000</t>
@@ -224,7 +226,7 @@
     <t>CIC.N0000</t>
   </si>
   <si>
-    <t>AEL.N0000</t>
+    <t>JXG.N0000</t>
   </si>
   <si>
     <t>🇱🇰   CSE STOCK MARKET TREND ANALYZER</t>
@@ -321,9 +323,6 @@
     <t>📂  WHAT EACH SHEET DOES</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>📋 HOW IT WORKS</t>
   </si>
   <si>
@@ -481,6 +480,9 @@
   </si>
   <si>
     <t>Close (LKR)</t>
+  </si>
+  <si>
+    <t>Volume</t>
   </si>
   <si>
     <t>Trading date (YYYY-MM-DD)</t>
@@ -1007,7 +1009,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;\(#,##0.00\);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="38" x14ac:knownFonts="1">
+  <fonts count="40" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1208,6 +1210,17 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF375623"/>
       <name val="Arial"/>
     </font>
@@ -1252,7 +1265,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1357,6 +1370,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
         <bgColor rgb="FFFFC7CE"/>
       </patternFill>
@@ -1386,7 +1405,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1424,11 +1443,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -1518,106 +1552,10 @@
     <xf numFmtId="0" fontId="20" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="25" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="30" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="30" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="24" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="4" fontId="25" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="32" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="32" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="24" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="24" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="36" fillId="21" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="24" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="37" fillId="22" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="24" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="36" fillId="17" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="24" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="37" fillId="18" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="24" fillId="16" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="24" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1626,6 +1564,117 @@
     <xf numFmtId="164" fontId="24" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="31" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="32" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="32" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="31" fillId="18" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="34" fillId="19" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="34" fillId="19" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="18" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="22" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="30" fillId="22" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="38" fillId="22" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="23" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="30" fillId="23" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="39" fillId="23" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="30" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="38" fillId="17" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="30" fillId="19" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="39" fillId="19" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="30" fillId="16" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="30" fillId="18" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="17" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="26" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1633,19 +1682,19 @@
     <xf numFmtId="0" fontId="27" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="35" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="36" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="37" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1686,15 +1735,15 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1904,8 +1953,8 @@
               <a:noFill/>
               <a:ln>
                 <a:noFill/>
+                <a:prstDash val="solid"/>
               </a:ln>
-              <a:effectLst/>
             </c:spPr>
             <c:txPr>
               <a:bodyPr/>
@@ -2334,7 +2383,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-6F67-4A43-8FD2-7318AFED7BF5}"/>
+              <c16:uniqueId val="{00000000-0024-4B73-B595-22E025BCAE8A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2369,8 +2418,8 @@
               <a:noFill/>
               <a:ln>
                 <a:noFill/>
+                <a:prstDash val="solid"/>
               </a:ln>
-              <a:effectLst/>
             </c:spPr>
             <c:txPr>
               <a:bodyPr/>
@@ -2799,7 +2848,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-6F67-4A43-8FD2-7318AFED7BF5}"/>
+              <c16:uniqueId val="{00000001-0024-4B73-B595-22E025BCAE8A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2834,8 +2883,8 @@
               <a:noFill/>
               <a:ln>
                 <a:noFill/>
+                <a:prstDash val="solid"/>
               </a:ln>
-              <a:effectLst/>
             </c:spPr>
             <c:txPr>
               <a:bodyPr/>
@@ -3225,7 +3274,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-6F67-4A43-8FD2-7318AFED7BF5}"/>
+              <c16:uniqueId val="{00000002-0024-4B73-B595-22E025BCAE8A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3541,8 +3590,8 @@
               <a:noFill/>
               <a:ln>
                 <a:noFill/>
+                <a:prstDash val="solid"/>
               </a:ln>
-              <a:effectLst/>
             </c:spPr>
             <c:txPr>
               <a:bodyPr/>
@@ -3971,7 +4020,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-99FE-45B2-9A1A-2106A77006BD}"/>
+              <c16:uniqueId val="{00000000-579A-4742-91EF-024C2463978B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4445,290 +4494,290 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="42" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="67" t="s">
+      <c r="B1" s="72" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
     </row>
     <row r="2" spans="2:8" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="69" t="s">
+      <c r="B2" s="74" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
     </row>
     <row r="3" spans="2:8" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="31" t="s">
+      <c r="B3" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="31" t="s">
+      <c r="C3" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="31" t="s">
+      <c r="D3" s="35" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="31" t="s">
+      <c r="E3" s="35" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="31" t="s">
+      <c r="F3" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="31" t="s">
+      <c r="H3" s="35" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="34">
-        <v>208</v>
-      </c>
-      <c r="E4" s="35">
-        <v>2.75</v>
-      </c>
-      <c r="F4" s="36">
-        <v>1.339829476248477E-2</v>
-      </c>
-      <c r="G4" s="37">
-        <v>323619109424</v>
-      </c>
-      <c r="H4" s="38" t="s">
+      <c r="D4" s="38">
+        <v>207.75</v>
+      </c>
+      <c r="E4" s="39">
+        <v>2.5</v>
+      </c>
+      <c r="F4" s="40">
+        <v>1.2180267965895251E-2</v>
+      </c>
+      <c r="G4" s="41">
+        <v>323230144148.25</v>
+      </c>
+      <c r="H4" s="42" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="39" t="s">
+      <c r="B5" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="C5" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="41">
-        <v>555</v>
-      </c>
-      <c r="E5" s="42">
-        <v>-0.25</v>
-      </c>
-      <c r="F5" s="43">
-        <v>-4.5024763619990998E-2</v>
-      </c>
-      <c r="G5" s="44">
-        <v>263736000000</v>
-      </c>
-      <c r="H5" s="45" t="s">
+      <c r="D5" s="45">
+        <v>550</v>
+      </c>
+      <c r="E5" s="46">
+        <v>-5.25</v>
+      </c>
+      <c r="F5" s="47">
+        <v>-0.94552003601981094</v>
+      </c>
+      <c r="G5" s="48">
+        <v>261360000000</v>
+      </c>
+      <c r="H5" s="49" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="36" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="33" t="s">
+      <c r="C6" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="34">
-        <v>42</v>
-      </c>
-      <c r="E6" s="35">
-        <v>0.4</v>
-      </c>
-      <c r="F6" s="36">
-        <v>0.96153846153846156</v>
-      </c>
-      <c r="G6" s="37">
-        <v>386414069748</v>
-      </c>
-      <c r="H6" s="38" t="s">
+      <c r="D6" s="38">
+        <v>42.5</v>
+      </c>
+      <c r="E6" s="39">
+        <v>0.9</v>
+      </c>
+      <c r="F6" s="40">
+        <v>2.1634615384615381E-2</v>
+      </c>
+      <c r="G6" s="41">
+        <v>391014237245</v>
+      </c>
+      <c r="H6" s="42" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="39" t="s">
+      <c r="B7" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="40" t="s">
+      <c r="C7" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="41">
-        <v>20.100000000000001</v>
-      </c>
-      <c r="E7" s="35">
-        <v>0</v>
-      </c>
-      <c r="F7" s="36">
-        <v>0</v>
-      </c>
-      <c r="G7" s="44">
-        <v>355948122501.59998</v>
-      </c>
-      <c r="H7" s="45" t="s">
+      <c r="D7" s="45">
+        <v>20.2</v>
+      </c>
+      <c r="E7" s="39">
+        <v>0.1</v>
+      </c>
+      <c r="F7" s="40">
+        <v>0.49751243781094528</v>
+      </c>
+      <c r="G7" s="48">
+        <v>357719008683.20001</v>
+      </c>
+      <c r="H7" s="49" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="34">
-        <v>399</v>
-      </c>
-      <c r="E8" s="42">
+      <c r="D8" s="38">
+        <v>397</v>
+      </c>
+      <c r="E8" s="46">
+        <v>-3</v>
+      </c>
+      <c r="F8" s="47">
+        <v>-0.75</v>
+      </c>
+      <c r="G8" s="41">
+        <v>182706617460</v>
+      </c>
+      <c r="H8" s="42" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="44" t="s">
+        <v>21</v>
+      </c>
+      <c r="D9" s="45">
+        <v>142</v>
+      </c>
+      <c r="E9" s="46">
         <v>-1</v>
       </c>
-      <c r="F8" s="43">
-        <v>-0.25</v>
-      </c>
-      <c r="G8" s="37">
-        <v>183627053820</v>
-      </c>
-      <c r="H8" s="38" t="s">
+      <c r="F9" s="47">
+        <v>-0.69930069930069927</v>
+      </c>
+      <c r="G9" s="48">
+        <v>166523507920</v>
+      </c>
+      <c r="H9" s="49" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="D9" s="41">
-        <v>142.75</v>
-      </c>
-      <c r="E9" s="42">
-        <v>-0.25</v>
-      </c>
-      <c r="F9" s="43">
-        <v>-0.17482517482517479</v>
-      </c>
-      <c r="G9" s="44">
-        <v>167403033490</v>
-      </c>
-      <c r="H9" s="45" t="s">
+    <row r="10" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="38">
+        <v>322</v>
+      </c>
+      <c r="E10" s="39">
+        <v>4</v>
+      </c>
+      <c r="F10" s="40">
+        <v>1.257861635220126E-2</v>
+      </c>
+      <c r="G10" s="41">
+        <v>92894278456</v>
+      </c>
+      <c r="H10" s="42" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="32" t="s">
-        <v>22</v>
-      </c>
-      <c r="C10" s="33" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="34">
-        <v>321</v>
-      </c>
-      <c r="E10" s="35">
-        <v>3</v>
-      </c>
-      <c r="F10" s="36">
-        <v>0.94339622641509435</v>
-      </c>
-      <c r="G10" s="37">
-        <v>92605786908</v>
-      </c>
-      <c r="H10" s="38" t="s">
+    <row r="11" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="45">
+        <v>463.5</v>
+      </c>
+      <c r="E11" s="39">
+        <v>3.5</v>
+      </c>
+      <c r="F11" s="40">
+        <v>0.76086956521739135</v>
+      </c>
+      <c r="G11" s="48">
+        <v>27810000000</v>
+      </c>
+      <c r="H11" s="49" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11" s="40" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="41">
-        <v>461</v>
-      </c>
-      <c r="E11" s="35">
-        <v>1</v>
-      </c>
-      <c r="F11" s="36">
-        <v>0.21739130434782611</v>
-      </c>
-      <c r="G11" s="44">
-        <v>27660000000</v>
-      </c>
-      <c r="H11" s="45" t="s">
+    <row r="12" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="36" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="37" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="38">
+        <v>1824.5</v>
+      </c>
+      <c r="E12" s="46">
+        <v>-5.25</v>
+      </c>
+      <c r="F12" s="47">
+        <v>-0.28692444322994942</v>
+      </c>
+      <c r="G12" s="41">
+        <v>341772183699.5</v>
+      </c>
+      <c r="H12" s="42" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="32" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="34">
-        <v>1828</v>
-      </c>
-      <c r="E12" s="42">
-        <v>-1.75</v>
-      </c>
-      <c r="F12" s="43">
-        <v>-9.5641481076649812E-2</v>
-      </c>
-      <c r="G12" s="37">
-        <v>342427816828</v>
-      </c>
-      <c r="H12" s="38" t="s">
+    <row r="13" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="43" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="44" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" s="45">
+        <v>800.75</v>
+      </c>
+      <c r="E13" s="39">
+        <v>0.75</v>
+      </c>
+      <c r="F13" s="40">
+        <v>9.375E-2</v>
+      </c>
+      <c r="G13" s="48">
+        <v>157256821385.5</v>
+      </c>
+      <c r="H13" s="49" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="2:8" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="39" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" s="40" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" s="41">
-        <v>820</v>
-      </c>
-      <c r="E13" s="35">
-        <v>20</v>
-      </c>
-      <c r="F13" s="36">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="G13" s="44">
-        <v>161037269480</v>
-      </c>
-      <c r="H13" s="45" t="s">
-        <v>11</v>
-      </c>
-    </row>
     <row r="15" spans="2:8" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="70" t="s">
+      <c r="B15" s="75" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="68"/>
-      <c r="D15" s="68"/>
-      <c r="E15" s="68"/>
-      <c r="F15" s="68"/>
-      <c r="G15" s="68"/>
-      <c r="H15" s="68"/>
+      <c r="C15" s="73"/>
+      <c r="D15" s="73"/>
+      <c r="E15" s="73"/>
+      <c r="F15" s="73"/>
+      <c r="G15" s="73"/>
+      <c r="H15" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4751,7 +4800,8 @@
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="5" width="13" customWidth="1"/>
+    <col min="4" max="4" width="25" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="3" customWidth="1"/>
     <col min="7" max="7" width="16" customWidth="1"/>
     <col min="8" max="8" width="28" customWidth="1"/>
@@ -4759,420 +4809,480 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="73" t="s">
+      <c r="B1" s="78" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
     </row>
     <row r="2" spans="2:11" ht="7.95" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:11" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="74" t="s">
+      <c r="B3" s="79" t="s">
         <v>32</v>
       </c>
-      <c r="C3" s="68"/>
-      <c r="D3" s="68"/>
-      <c r="E3" s="68"/>
-      <c r="G3" s="72" t="s">
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="G3" s="77" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="68"/>
-      <c r="I3" s="68"/>
-      <c r="J3" s="68"/>
+      <c r="H3" s="73"/>
+      <c r="I3" s="73"/>
+      <c r="J3" s="73"/>
     </row>
     <row r="4" spans="2:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="50" t="s">
         <v>35</v>
       </c>
-      <c r="E4" s="46" t="s">
+      <c r="E4" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="47" t="s">
+      <c r="G4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="H4" s="47" t="s">
+      <c r="H4" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="I4" s="47" t="s">
+      <c r="I4" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="J4" s="47" t="s">
+      <c r="J4" s="51" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="52" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="49"/>
-      <c r="D5" s="50">
-        <v>0</v>
-      </c>
-      <c r="E5" s="51">
+      <c r="C5" s="66" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="53">
+        <v>0.6</v>
+      </c>
+      <c r="E5" s="54">
         <v>0.2</v>
       </c>
-      <c r="G5" s="52" t="s">
+      <c r="G5" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="53"/>
-      <c r="I5" s="54">
-        <v>0</v>
-      </c>
-      <c r="J5" s="55">
+      <c r="H5" s="67" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" s="56">
+        <v>742</v>
+      </c>
+      <c r="J5" s="57">
         <v>-9.7323600973236016E-2</v>
       </c>
     </row>
     <row r="6" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="56" t="s">
+      <c r="B6" s="58" t="s">
         <v>38</v>
       </c>
-      <c r="C6" s="57"/>
-      <c r="D6" s="58">
-        <v>0</v>
-      </c>
-      <c r="E6" s="59">
+      <c r="C6" s="68" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="59">
+        <v>1200</v>
+      </c>
+      <c r="E6" s="60">
         <v>0.1420413990007138</v>
       </c>
-      <c r="G6" s="60" t="s">
+      <c r="G6" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="H6" s="61"/>
+      <c r="H6" s="69" t="s">
+        <v>39</v>
+      </c>
       <c r="I6" s="62">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="J6" s="63">
-        <v>-4.1860465116279083E-2</v>
+        <v>-7.2164948453608255E-2</v>
       </c>
     </row>
     <row r="7" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="50">
-        <v>0</v>
-      </c>
-      <c r="E7" s="51">
-        <v>8.5802742149491365E-2</v>
-      </c>
-      <c r="G7" s="52" t="s">
+      <c r="C7" s="66" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="53">
+        <v>2019</v>
+      </c>
+      <c r="E7" s="54">
+        <v>0.12416481069042321</v>
+      </c>
+      <c r="G7" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="H7" s="53"/>
-      <c r="I7" s="54">
-        <v>0</v>
-      </c>
-      <c r="J7" s="55">
+      <c r="H7" s="67" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="56">
+        <v>48</v>
+      </c>
+      <c r="J7" s="57">
+        <v>-3.8076152304609208E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="58" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="68" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="59">
+        <v>614</v>
+      </c>
+      <c r="E8" s="60">
+        <v>8.6245024325519684E-2</v>
+      </c>
+      <c r="G8" s="61" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="69" t="s">
+        <v>43</v>
+      </c>
+      <c r="I8" s="62">
+        <v>4401.5</v>
+      </c>
+      <c r="J8" s="63">
         <v>-3.687089715536105E-2</v>
       </c>
     </row>
-    <row r="8" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="56" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="57"/>
-      <c r="D8" s="58">
-        <v>0</v>
-      </c>
-      <c r="E8" s="59">
+    <row r="9" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="66" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="53">
+        <v>170</v>
+      </c>
+      <c r="E9" s="54">
         <v>7.9365079365079361E-2</v>
       </c>
-      <c r="G8" s="60" t="s">
-        <v>43</v>
-      </c>
-      <c r="H8" s="61"/>
-      <c r="I8" s="62">
-        <v>0</v>
-      </c>
-      <c r="J8" s="63">
+      <c r="G9" s="55" t="s">
+        <v>45</v>
+      </c>
+      <c r="H9" s="67" t="s">
+        <v>45</v>
+      </c>
+      <c r="I9" s="56">
+        <v>2699</v>
+      </c>
+      <c r="J9" s="57">
         <v>-3.538241601143674E-2</v>
       </c>
     </row>
-    <row r="9" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="49"/>
-      <c r="D9" s="50">
-        <v>0</v>
-      </c>
-      <c r="E9" s="51">
+    <row r="10" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="58" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="68" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="59">
+        <v>2.8</v>
+      </c>
+      <c r="E10" s="60">
         <v>7.6923076923076927E-2</v>
       </c>
-      <c r="G9" s="52" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="53"/>
-      <c r="I9" s="54">
-        <v>0</v>
-      </c>
-      <c r="J9" s="55">
-        <v>-3.5087719298245612E-2</v>
-      </c>
-    </row>
-    <row r="10" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="56" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" s="57"/>
-      <c r="D10" s="58">
-        <v>0</v>
-      </c>
-      <c r="E10" s="59">
+      <c r="G10" s="61" t="s">
+        <v>47</v>
+      </c>
+      <c r="H10" s="69" t="s">
+        <v>47</v>
+      </c>
+      <c r="I10" s="62">
+        <v>22.8</v>
+      </c>
+      <c r="J10" s="63">
+        <v>-3.3898305084745763E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="52" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="66" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="53">
+        <v>162</v>
+      </c>
+      <c r="E11" s="54">
         <v>7.6411960132890366E-2</v>
       </c>
-      <c r="G10" s="60" t="s">
-        <v>47</v>
-      </c>
-      <c r="H10" s="61"/>
-      <c r="I10" s="62">
-        <v>0</v>
-      </c>
-      <c r="J10" s="63">
+      <c r="G11" s="55" t="s">
+        <v>49</v>
+      </c>
+      <c r="H11" s="67" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="56">
+        <v>44.3</v>
+      </c>
+      <c r="J11" s="57">
+        <v>-3.2751091703056769E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="58" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="68" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="59">
+        <v>9.9</v>
+      </c>
+      <c r="E12" s="60">
+        <v>7.6086956521739135E-2</v>
+      </c>
+      <c r="G12" s="61" t="s">
+        <v>51</v>
+      </c>
+      <c r="H12" s="69" t="s">
+        <v>51</v>
+      </c>
+      <c r="I12" s="62">
+        <v>148.25</v>
+      </c>
+      <c r="J12" s="63">
+        <v>-3.1045751633986929E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="52" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="66" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="53">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="E13" s="54">
+        <v>7.301587301587302E-2</v>
+      </c>
+      <c r="G13" s="55" t="s">
+        <v>53</v>
+      </c>
+      <c r="H13" s="67" t="s">
+        <v>53</v>
+      </c>
+      <c r="I13" s="56">
+        <v>13</v>
+      </c>
+      <c r="J13" s="57">
         <v>-2.9850746268656719E-2</v>
       </c>
     </row>
-    <row r="11" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="49"/>
-      <c r="D11" s="50">
-        <v>0</v>
-      </c>
-      <c r="E11" s="51">
-        <v>7.6086956521739135E-2</v>
-      </c>
-      <c r="G11" s="52" t="s">
-        <v>49</v>
-      </c>
-      <c r="H11" s="53"/>
-      <c r="I11" s="54">
-        <v>0</v>
-      </c>
-      <c r="J11" s="55">
-        <v>-2.7472527472527469E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="56" t="s">
+    <row r="14" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="58" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" s="68" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="59">
+        <v>510</v>
+      </c>
+      <c r="E14" s="60">
+        <v>6.416275430359937E-2</v>
+      </c>
+      <c r="G14" s="61" t="s">
+        <v>55</v>
+      </c>
+      <c r="H14" s="69" t="s">
+        <v>55</v>
+      </c>
+      <c r="I14" s="62">
+        <v>310</v>
+      </c>
+      <c r="J14" s="63">
+        <v>-2.7450980392156859E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="76" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="73"/>
+      <c r="D17" s="73"/>
+      <c r="E17" s="73"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B18" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="C18" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="35" t="s">
+        <v>57</v>
+      </c>
+      <c r="E18" s="35" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="70" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="64">
+        <v>70325287.25</v>
+      </c>
+      <c r="E19" s="41">
+        <v>493773</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="C12" s="57"/>
-      <c r="D12" s="58">
-        <v>0</v>
-      </c>
-      <c r="E12" s="59">
-        <v>7.301587301587302E-2</v>
-      </c>
-      <c r="G12" s="60" t="s">
-        <v>51</v>
-      </c>
-      <c r="H12" s="61"/>
-      <c r="I12" s="62">
-        <v>0</v>
-      </c>
-      <c r="J12" s="63">
-        <v>-2.7450980392156859E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="48" t="s">
-        <v>52</v>
-      </c>
-      <c r="C13" s="49"/>
-      <c r="D13" s="50">
-        <v>0</v>
-      </c>
-      <c r="E13" s="51">
-        <v>6.8965517241379309E-2</v>
-      </c>
-      <c r="G13" s="52" t="s">
-        <v>53</v>
-      </c>
-      <c r="H13" s="53"/>
-      <c r="I13" s="54">
-        <v>0</v>
-      </c>
-      <c r="J13" s="55">
-        <v>-2.684563758389262E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="56" t="s">
-        <v>54</v>
-      </c>
-      <c r="C14" s="57"/>
-      <c r="D14" s="58">
-        <v>0</v>
-      </c>
-      <c r="E14" s="59">
-        <v>6.5652522017614096E-2</v>
-      </c>
-      <c r="G14" s="60" t="s">
-        <v>55</v>
-      </c>
-      <c r="H14" s="61"/>
-      <c r="I14" s="62">
-        <v>0</v>
-      </c>
-      <c r="J14" s="63">
-        <v>-2.542372881355932E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="71" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="68"/>
-      <c r="D17" s="68"/>
-      <c r="E17" s="68"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B18" s="31" t="s">
-        <v>2</v>
-      </c>
-      <c r="C18" s="31" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="31" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="31" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="19" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="32" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="33"/>
-      <c r="D19" s="64">
-        <v>0</v>
-      </c>
-      <c r="E19" s="37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="40"/>
+      <c r="C20" s="71" t="s">
+        <v>50</v>
+      </c>
       <c r="D20" s="65">
-        <v>0</v>
-      </c>
-      <c r="E20" s="44">
-        <v>0</v>
+        <v>3673911364.3000002</v>
+      </c>
+      <c r="E20" s="48">
+        <v>415671066</v>
       </c>
     </row>
     <row r="21" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="32" t="s">
+      <c r="B21" s="36" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="33"/>
+      <c r="C21" s="70" t="s">
+        <v>16</v>
+      </c>
       <c r="D21" s="64">
-        <v>0</v>
-      </c>
-      <c r="E21" s="37">
-        <v>0</v>
+        <v>125921099.3</v>
+      </c>
+      <c r="E21" s="41">
+        <v>6294593</v>
       </c>
     </row>
     <row r="22" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="39" t="s">
+      <c r="B22" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="40"/>
+      <c r="C22" s="71" t="s">
+        <v>14</v>
+      </c>
       <c r="D22" s="65">
-        <v>0</v>
-      </c>
-      <c r="E22" s="44">
-        <v>0</v>
+        <v>87232180.099999994</v>
+      </c>
+      <c r="E22" s="48">
+        <v>2083956</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="32" t="s">
-        <v>58</v>
-      </c>
-      <c r="C23" s="33"/>
+      <c r="B23" s="36" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="70" t="s">
+        <v>18</v>
+      </c>
       <c r="D23" s="64">
-        <v>0</v>
-      </c>
-      <c r="E23" s="37">
-        <v>0</v>
+        <v>368530992.75</v>
+      </c>
+      <c r="E23" s="41">
+        <v>932337</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="39" t="s">
+      <c r="B24" s="43" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="40"/>
+      <c r="C24" s="71" t="s">
+        <v>59</v>
+      </c>
       <c r="D24" s="65">
-        <v>0</v>
-      </c>
-      <c r="E24" s="44">
-        <v>0</v>
+        <v>19035227.699999999</v>
+      </c>
+      <c r="E24" s="48">
+        <v>768339</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="33"/>
+      <c r="C25" s="70" t="s">
+        <v>9</v>
+      </c>
       <c r="D25" s="64">
-        <v>0</v>
-      </c>
-      <c r="E25" s="37">
-        <v>0</v>
+        <v>228658096.5</v>
+      </c>
+      <c r="E25" s="41">
+        <v>1102473</v>
       </c>
     </row>
     <row r="26" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="39" t="s">
+      <c r="B26" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="40"/>
+      <c r="C26" s="71" t="s">
+        <v>60</v>
+      </c>
       <c r="D26" s="65">
-        <v>0</v>
-      </c>
-      <c r="E26" s="44">
-        <v>0</v>
+        <v>36524430</v>
+      </c>
+      <c r="E26" s="48">
+        <v>4029260</v>
       </c>
     </row>
     <row r="27" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="33"/>
+      <c r="B27" s="36" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="70" t="s">
+        <v>61</v>
+      </c>
       <c r="D27" s="64">
-        <v>0</v>
-      </c>
-      <c r="E27" s="37">
-        <v>0</v>
+        <v>88954282.299999997</v>
+      </c>
+      <c r="E27" s="41">
+        <v>2694895</v>
       </c>
     </row>
     <row r="28" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="39" t="s">
-        <v>61</v>
-      </c>
-      <c r="C28" s="40"/>
+      <c r="B28" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="71" t="s">
+        <v>62</v>
+      </c>
       <c r="D28" s="65">
-        <v>0</v>
-      </c>
-      <c r="E28" s="44">
-        <v>0</v>
+        <v>31091235.800000001</v>
+      </c>
+      <c r="E28" s="48">
+        <v>2394854</v>
       </c>
     </row>
   </sheetData>
@@ -5202,184 +5312,182 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="51.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="78" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
+      <c r="B1" s="83" t="s">
+        <v>63</v>
+      </c>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
     </row>
     <row r="2" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="89" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
+      <c r="B2" s="98" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
     </row>
     <row r="3" spans="2:4" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="86" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
+      <c r="B4" s="91" t="s">
+        <v>65</v>
+      </c>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
     </row>
     <row r="5" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="88" t="s">
-        <v>65</v>
-      </c>
-      <c r="C5" s="68"/>
-      <c r="D5" s="68"/>
+      <c r="B5" s="93" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
     </row>
     <row r="6" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="79" t="s">
-        <v>66</v>
-      </c>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
+      <c r="B6" s="84" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="73"/>
+      <c r="D6" s="73"/>
     </row>
     <row r="7" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="88" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
+      <c r="B7" s="93" t="s">
+        <v>68</v>
+      </c>
+      <c r="C7" s="73"/>
+      <c r="D7" s="73"/>
     </row>
     <row r="8" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="79" t="s">
-        <v>68</v>
-      </c>
-      <c r="C8" s="68"/>
-      <c r="D8" s="68"/>
+      <c r="B8" s="84" t="s">
+        <v>69</v>
+      </c>
+      <c r="C8" s="73"/>
+      <c r="D8" s="73"/>
     </row>
     <row r="9" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="88" t="s">
-        <v>69</v>
-      </c>
-      <c r="C9" s="68"/>
-      <c r="D9" s="68"/>
+      <c r="B9" s="93" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="73"/>
+      <c r="D9" s="73"/>
     </row>
     <row r="10" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="79" t="s">
-        <v>70</v>
-      </c>
-      <c r="C10" s="68"/>
-      <c r="D10" s="68"/>
+      <c r="B10" s="84" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="73"/>
+      <c r="D10" s="73"/>
     </row>
     <row r="11" spans="2:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="81" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" s="68"/>
-      <c r="D12" s="68"/>
+      <c r="B12" s="86" t="s">
+        <v>72</v>
+      </c>
+      <c r="C12" s="73"/>
+      <c r="D12" s="73"/>
     </row>
     <row r="13" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="85" t="s">
-        <v>72</v>
+      <c r="B13" s="90" t="s">
+        <v>73</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="68"/>
+      <c r="B14" s="73"/>
       <c r="C14" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D14" s="4"/>
     </row>
     <row r="15" spans="2:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="85" t="s">
-        <v>76</v>
+      <c r="B16" s="90" t="s">
+        <v>77</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="68"/>
+      <c r="B17" s="73"/>
       <c r="C17" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D17" s="4"/>
     </row>
     <row r="18" spans="2:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="19" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="85" t="s">
-        <v>79</v>
+      <c r="B19" s="90" t="s">
+        <v>80</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="68"/>
+      <c r="B20" s="73"/>
       <c r="C20" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="21" spans="2:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="22" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="85" t="s">
-        <v>82</v>
+      <c r="B22" s="90" t="s">
+        <v>83</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="68"/>
+      <c r="B23" s="73"/>
       <c r="C23" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D23" s="4"/>
     </row>
     <row r="24" spans="2:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="93" t="s">
-        <v>85</v>
+      <c r="B25" s="97" t="s">
+        <v>86</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="68"/>
+      <c r="B26" s="73"/>
       <c r="C26" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D26" s="4"/>
     </row>
     <row r="27" spans="2:4" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="28" spans="2:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="81" t="s">
-        <v>89</v>
-      </c>
-      <c r="C29" s="68"/>
-      <c r="D29" s="68"/>
+      <c r="B29" s="86" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="73"/>
+      <c r="D29" s="73"/>
     </row>
     <row r="30" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="91" t="s">
-        <v>90</v>
-      </c>
+      <c r="B30" s="95"/>
       <c r="C30" s="5" t="s">
         <v>91</v>
       </c>
@@ -5388,17 +5496,15 @@
       </c>
     </row>
     <row r="31" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="68"/>
-      <c r="C31" s="75" t="s">
+      <c r="B31" s="73"/>
+      <c r="C31" s="80" t="s">
         <v>93</v>
       </c>
-      <c r="D31" s="68"/>
+      <c r="D31" s="73"/>
     </row>
     <row r="32" spans="2:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="33" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="90" t="s">
-        <v>90</v>
-      </c>
+      <c r="B33" s="94"/>
       <c r="C33" s="7" t="s">
         <v>94</v>
       </c>
@@ -5407,17 +5513,15 @@
       </c>
     </row>
     <row r="34" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="68"/>
-      <c r="C34" s="75" t="s">
+      <c r="B34" s="73"/>
+      <c r="C34" s="80" t="s">
         <v>96</v>
       </c>
-      <c r="D34" s="68"/>
+      <c r="D34" s="73"/>
     </row>
     <row r="35" spans="2:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="36" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="82" t="s">
-        <v>90</v>
-      </c>
+      <c r="B36" s="87"/>
       <c r="C36" s="9" t="s">
         <v>97</v>
       </c>
@@ -5426,17 +5530,15 @@
       </c>
     </row>
     <row r="37" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="68"/>
-      <c r="C37" s="75" t="s">
+      <c r="B37" s="73"/>
+      <c r="C37" s="80" t="s">
         <v>98</v>
       </c>
-      <c r="D37" s="68"/>
+      <c r="D37" s="73"/>
     </row>
     <row r="38" spans="2:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="39" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="83" t="s">
-        <v>90</v>
-      </c>
+      <c r="B39" s="88"/>
       <c r="C39" s="11" t="s">
         <v>99</v>
       </c>
@@ -5445,17 +5547,15 @@
       </c>
     </row>
     <row r="40" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="68"/>
-      <c r="C40" s="75" t="s">
+      <c r="B40" s="73"/>
+      <c r="C40" s="80" t="s">
         <v>101</v>
       </c>
-      <c r="D40" s="68"/>
+      <c r="D40" s="73"/>
     </row>
     <row r="41" spans="2:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="42" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="82" t="s">
-        <v>90</v>
-      </c>
+      <c r="B42" s="87"/>
       <c r="C42" s="9" t="s">
         <v>102</v>
       </c>
@@ -5464,17 +5564,15 @@
       </c>
     </row>
     <row r="43" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="68"/>
-      <c r="C43" s="75" t="s">
+      <c r="B43" s="73"/>
+      <c r="C43" s="80" t="s">
         <v>104</v>
       </c>
-      <c r="D43" s="68"/>
+      <c r="D43" s="73"/>
     </row>
     <row r="44" spans="2:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="45" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="90" t="s">
-        <v>90</v>
-      </c>
+      <c r="B45" s="94"/>
       <c r="C45" s="7" t="s">
         <v>105</v>
       </c>
@@ -5483,168 +5581,168 @@
       </c>
     </row>
     <row r="46" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="68"/>
-      <c r="C46" s="75" t="s">
+      <c r="B46" s="73"/>
+      <c r="C46" s="80" t="s">
         <v>107</v>
       </c>
-      <c r="D46" s="68"/>
+      <c r="D46" s="73"/>
     </row>
     <row r="47" spans="2:4" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="48" spans="2:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="49" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="86" t="s">
+      <c r="B49" s="91" t="s">
         <v>108</v>
       </c>
-      <c r="C49" s="68"/>
-      <c r="D49" s="68"/>
+      <c r="C49" s="73"/>
+      <c r="D49" s="73"/>
     </row>
     <row r="50" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="C50" s="84" t="s">
+      <c r="C50" s="89" t="s">
         <v>110</v>
       </c>
-      <c r="D50" s="68"/>
+      <c r="D50" s="73"/>
     </row>
     <row r="51" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="C51" s="84" t="s">
+      <c r="C51" s="89" t="s">
         <v>112</v>
       </c>
-      <c r="D51" s="68"/>
+      <c r="D51" s="73"/>
     </row>
     <row r="52" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="C52" s="84" t="s">
+      <c r="C52" s="89" t="s">
         <v>114</v>
       </c>
-      <c r="D52" s="68"/>
+      <c r="D52" s="73"/>
     </row>
     <row r="53" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="13" t="s">
         <v>115</v>
       </c>
-      <c r="C53" s="84" t="s">
+      <c r="C53" s="89" t="s">
         <v>116</v>
       </c>
-      <c r="D53" s="68"/>
+      <c r="D53" s="73"/>
     </row>
     <row r="54" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="13" t="s">
         <v>117</v>
       </c>
-      <c r="C54" s="84" t="s">
+      <c r="C54" s="89" t="s">
         <v>118</v>
       </c>
-      <c r="D54" s="68"/>
+      <c r="D54" s="73"/>
     </row>
     <row r="55" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="14"/>
-      <c r="C55" s="87" t="s">
+      <c r="C55" s="92" t="s">
         <v>119</v>
       </c>
-      <c r="D55" s="68"/>
+      <c r="D55" s="73"/>
     </row>
     <row r="56" spans="2:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="57" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B57" s="80" t="s">
+      <c r="B57" s="85" t="s">
         <v>120</v>
       </c>
-      <c r="C57" s="68"/>
-      <c r="D57" s="68"/>
+      <c r="C57" s="73"/>
+      <c r="D57" s="73"/>
     </row>
     <row r="58" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B58" s="76" t="s">
+      <c r="B58" s="81" t="s">
         <v>121</v>
       </c>
-      <c r="C58" s="68"/>
-      <c r="D58" s="68"/>
+      <c r="C58" s="73"/>
+      <c r="D58" s="73"/>
     </row>
     <row r="59" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="76" t="s">
+      <c r="B59" s="81" t="s">
         <v>122</v>
       </c>
-      <c r="C59" s="68"/>
-      <c r="D59" s="68"/>
+      <c r="C59" s="73"/>
+      <c r="D59" s="73"/>
     </row>
     <row r="60" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="76" t="s">
+      <c r="B60" s="81" t="s">
         <v>123</v>
       </c>
-      <c r="C60" s="68"/>
-      <c r="D60" s="68"/>
+      <c r="C60" s="73"/>
+      <c r="D60" s="73"/>
     </row>
     <row r="61" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="76" t="s">
+      <c r="B61" s="81" t="s">
         <v>124</v>
       </c>
-      <c r="C61" s="68"/>
-      <c r="D61" s="68"/>
+      <c r="C61" s="73"/>
+      <c r="D61" s="73"/>
     </row>
     <row r="62" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B62" s="76" t="s">
+      <c r="B62" s="81" t="s">
         <v>125</v>
       </c>
-      <c r="C62" s="68"/>
-      <c r="D62" s="68"/>
+      <c r="C62" s="73"/>
+      <c r="D62" s="73"/>
     </row>
     <row r="63" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="76" t="s">
+      <c r="B63" s="81" t="s">
         <v>126</v>
       </c>
-      <c r="C63" s="68"/>
-      <c r="D63" s="68"/>
+      <c r="C63" s="73"/>
+      <c r="D63" s="73"/>
     </row>
     <row r="64" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B64" s="76" t="s">
+      <c r="B64" s="81" t="s">
         <v>127</v>
       </c>
-      <c r="C64" s="68"/>
-      <c r="D64" s="68"/>
+      <c r="C64" s="73"/>
+      <c r="D64" s="73"/>
     </row>
     <row r="65" spans="2:4" ht="13.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" spans="2:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B66" s="92" t="s">
+      <c r="B66" s="96" t="s">
         <v>128</v>
       </c>
-      <c r="C66" s="68"/>
-      <c r="D66" s="68"/>
+      <c r="C66" s="73"/>
+      <c r="D66" s="73"/>
     </row>
     <row r="67" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="C67" s="77" t="s">
+      <c r="C67" s="82" t="s">
         <v>130</v>
       </c>
-      <c r="D67" s="68"/>
+      <c r="D67" s="73"/>
     </row>
     <row r="68" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="C68" s="77" t="s">
+      <c r="C68" s="82" t="s">
         <v>132</v>
       </c>
-      <c r="D68" s="68"/>
+      <c r="D68" s="73"/>
     </row>
     <row r="69" spans="2:4" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="C69" s="77" t="s">
+      <c r="C69" s="82" t="s">
         <v>134</v>
       </c>
-      <c r="D69" s="68"/>
+      <c r="D69" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="B66:D66"/>
     <mergeCell ref="C67:D67"/>
     <mergeCell ref="B22:B23"/>
@@ -5652,15 +5750,6 @@
     <mergeCell ref="B58:D58"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="C53:D53"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="C43:D43"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="C46:D46"/>
-    <mergeCell ref="B63:D63"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C51:D51"/>
-    <mergeCell ref="B33:B34"/>
-    <mergeCell ref="B12:D12"/>
     <mergeCell ref="C52:D52"/>
     <mergeCell ref="B62:D62"/>
     <mergeCell ref="B7:D7"/>
@@ -5668,13 +5757,22 @@
     <mergeCell ref="B45:B46"/>
     <mergeCell ref="B59:D59"/>
     <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C69:D69"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B49:D49"/>
+    <mergeCell ref="C55:D55"/>
     <mergeCell ref="C50:D50"/>
-    <mergeCell ref="B2:D2"/>
     <mergeCell ref="C40:D40"/>
     <mergeCell ref="C31:D31"/>
-    <mergeCell ref="B6:D6"/>
     <mergeCell ref="B19:B20"/>
-    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C46:D46"/>
+    <mergeCell ref="B63:D63"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C51:D51"/>
+    <mergeCell ref="B33:B34"/>
     <mergeCell ref="C34:D34"/>
     <mergeCell ref="B60:D60"/>
     <mergeCell ref="C68:D68"/>
@@ -5686,11 +5784,11 @@
     <mergeCell ref="B42:B43"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="B39:B40"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="B49:D49"/>
-    <mergeCell ref="C55:D55"/>
     <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B12:D12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5713,54 +5811,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="81" t="s">
+      <c r="B1" s="86" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
     </row>
     <row r="2" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="94" t="s">
+      <c r="B2" s="99" t="s">
         <v>136</v>
       </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
     </row>
     <row r="3" spans="2:7" ht="33" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="66" t="s">
+      <c r="B3" s="34" t="s">
         <v>137</v>
       </c>
-      <c r="C3" s="65">
+      <c r="C3" s="33">
         <v>207</v>
       </c>
-      <c r="D3" s="65">
+      <c r="D3" s="33">
         <v>208.25</v>
       </c>
-      <c r="E3" s="65">
+      <c r="E3" s="33">
         <v>206</v>
       </c>
-      <c r="F3" s="41">
+      <c r="F3" s="31">
         <v>208</v>
       </c>
-      <c r="G3" s="44">
+      <c r="G3" s="32">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="95" t="s">
+      <c r="B4" s="100" t="s">
         <v>138</v>
       </c>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
     </row>
     <row r="5" spans="2:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="16" t="s">
@@ -5779,32 +5877,32 @@
         <v>143</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>57</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="18" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C7" s="19">
         <v>199.9</v>
@@ -5824,7 +5922,7 @@
     </row>
     <row r="8" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="21" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C8" s="22">
         <v>199.89</v>
@@ -5844,7 +5942,7 @@
     </row>
     <row r="9" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="18" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C9" s="19">
         <v>197.67</v>
@@ -5864,7 +5962,7 @@
     </row>
     <row r="10" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C10" s="22">
         <v>198.36</v>
@@ -5884,7 +5982,7 @@
     </row>
     <row r="11" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="18" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C11" s="19">
         <v>195.57</v>
@@ -5904,7 +6002,7 @@
     </row>
     <row r="12" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="21" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C12" s="22">
         <v>196.91</v>
@@ -5924,7 +6022,7 @@
     </row>
     <row r="13" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="18" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C13" s="19">
         <v>195.62</v>
@@ -5944,7 +6042,7 @@
     </row>
     <row r="14" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="21" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C14" s="22">
         <v>197.2</v>
@@ -5964,7 +6062,7 @@
     </row>
     <row r="15" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C15" s="19">
         <v>198.83</v>
@@ -5984,7 +6082,7 @@
     </row>
     <row r="16" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C16" s="22">
         <v>199.13</v>
@@ -6004,7 +6102,7 @@
     </row>
     <row r="17" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="18" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C17" s="19">
         <v>200.21</v>
@@ -6024,7 +6122,7 @@
     </row>
     <row r="18" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="21" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C18" s="22">
         <v>199.81</v>
@@ -6044,7 +6142,7 @@
     </row>
     <row r="19" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="18" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C19" s="19">
         <v>197.63</v>
@@ -6064,7 +6162,7 @@
     </row>
     <row r="20" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="21" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C20" s="22">
         <v>200.55</v>
@@ -6084,7 +6182,7 @@
     </row>
     <row r="21" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="18" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C21" s="19">
         <v>199.11</v>
@@ -6104,7 +6202,7 @@
     </row>
     <row r="22" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="21" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C22" s="22">
         <v>200.92</v>
@@ -6124,7 +6222,7 @@
     </row>
     <row r="23" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="18" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C23" s="19">
         <v>199.15</v>
@@ -6144,7 +6242,7 @@
     </row>
     <row r="24" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="21" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C24" s="22">
         <v>198.5</v>
@@ -6164,7 +6262,7 @@
     </row>
     <row r="25" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C25" s="19">
         <v>199.93</v>
@@ -6184,7 +6282,7 @@
     </row>
     <row r="26" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="21" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C26" s="22">
         <v>202.92</v>
@@ -6204,7 +6302,7 @@
     </row>
     <row r="27" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="18" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C27" s="19">
         <v>203.84</v>
@@ -6224,7 +6322,7 @@
     </row>
     <row r="28" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="21" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C28" s="22">
         <v>207.68</v>
@@ -6244,7 +6342,7 @@
     </row>
     <row r="29" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="18" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C29" s="19">
         <v>210.37</v>
@@ -6264,7 +6362,7 @@
     </row>
     <row r="30" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="21" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C30" s="22">
         <v>211.35</v>
@@ -6284,7 +6382,7 @@
     </row>
     <row r="31" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="18" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C31" s="19">
         <v>208.42</v>
@@ -6304,7 +6402,7 @@
     </row>
     <row r="32" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C32" s="22">
         <v>210.14</v>
@@ -6324,7 +6422,7 @@
     </row>
     <row r="33" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C33" s="19">
         <v>210.43</v>
@@ -6344,7 +6442,7 @@
     </row>
     <row r="34" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="21" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C34" s="22">
         <v>211.23</v>
@@ -6364,7 +6462,7 @@
     </row>
     <row r="35" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="18" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C35" s="19">
         <v>212.68</v>
@@ -6384,7 +6482,7 @@
     </row>
     <row r="36" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="21" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C36" s="22">
         <v>209.12</v>
@@ -6404,7 +6502,7 @@
     </row>
     <row r="37" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="18" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C37" s="19">
         <v>209.84</v>
@@ -6424,7 +6522,7 @@
     </row>
     <row r="38" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C38" s="22">
         <v>212.51</v>
@@ -6444,7 +6542,7 @@
     </row>
     <row r="39" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="18" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C39" s="19">
         <v>214.03</v>
@@ -6464,7 +6562,7 @@
     </row>
     <row r="40" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="21" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C40" s="22">
         <v>216.91</v>
@@ -6484,7 +6582,7 @@
     </row>
     <row r="41" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="18" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C41" s="19">
         <v>216.02</v>
@@ -6504,7 +6602,7 @@
     </row>
     <row r="42" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="21" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C42" s="22">
         <v>219.26</v>
@@ -6524,7 +6622,7 @@
     </row>
     <row r="43" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="18" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C43" s="19">
         <v>217.04</v>
@@ -6544,7 +6642,7 @@
     </row>
     <row r="44" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="21" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C44" s="22">
         <v>217.02</v>
@@ -6564,7 +6662,7 @@
     </row>
     <row r="45" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="18" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C45" s="19">
         <v>218.49</v>
@@ -6584,7 +6682,7 @@
     </row>
     <row r="46" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="21" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C46" s="22">
         <v>216.82</v>
@@ -6604,7 +6702,7 @@
     </row>
     <row r="47" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="18" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C47" s="19">
         <v>218.12</v>
@@ -6624,7 +6722,7 @@
     </row>
     <row r="48" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="21" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C48" s="22">
         <v>222.91</v>
@@ -6644,7 +6742,7 @@
     </row>
     <row r="49" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="18" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C49" s="19">
         <v>224.31</v>
@@ -6664,7 +6762,7 @@
     </row>
     <row r="50" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="21" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C50" s="22">
         <v>223.03</v>
@@ -6684,7 +6782,7 @@
     </row>
     <row r="51" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="18" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C51" s="19">
         <v>221.01</v>
@@ -6704,7 +6802,7 @@
     </row>
     <row r="52" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="21" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C52" s="22">
         <v>222.64</v>
@@ -6724,7 +6822,7 @@
     </row>
     <row r="53" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="18" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C53" s="19">
         <v>223.98</v>
@@ -6744,7 +6842,7 @@
     </row>
     <row r="54" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="21" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C54" s="22">
         <v>225.72</v>
@@ -6764,7 +6862,7 @@
     </row>
     <row r="55" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="18" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C55" s="19">
         <v>227.39</v>
@@ -6784,7 +6882,7 @@
     </row>
     <row r="56" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="21" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C56" s="22">
         <v>224.9</v>
@@ -6804,7 +6902,7 @@
     </row>
     <row r="57" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="18" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C57" s="19">
         <v>229.46</v>
@@ -6824,7 +6922,7 @@
     </row>
     <row r="58" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="21" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C58" s="22">
         <v>228.42</v>
@@ -6844,7 +6942,7 @@
     </row>
     <row r="59" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="18" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C59" s="19">
         <v>227.48</v>
@@ -6864,7 +6962,7 @@
     </row>
     <row r="60" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="21" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C60" s="22">
         <v>229.44</v>
@@ -6884,7 +6982,7 @@
     </row>
     <row r="61" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="18" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C61" s="19">
         <v>225.92</v>
@@ -6904,7 +7002,7 @@
     </row>
     <row r="62" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="21" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C62" s="22">
         <v>227.47</v>
@@ -6924,7 +7022,7 @@
     </row>
     <row r="63" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="18" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C63" s="19">
         <v>227.95</v>
@@ -6944,7 +7042,7 @@
     </row>
     <row r="64" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="21" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C64" s="22">
         <v>227.9</v>
@@ -6964,7 +7062,7 @@
     </row>
     <row r="65" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="18" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C65" s="19">
         <v>228.38</v>
@@ -6984,7 +7082,7 @@
     </row>
     <row r="66" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="21" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C66" s="22">
         <v>232.3</v>
@@ -7004,7 +7102,7 @@
     </row>
     <row r="67" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="18" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C67" s="19">
         <v>228.96</v>
@@ -7024,7 +7122,7 @@
     </row>
     <row r="68" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="21" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C68" s="22">
         <v>230.89</v>
@@ -7044,7 +7142,7 @@
     </row>
     <row r="69" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="18" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C69" s="19">
         <v>231.67</v>
@@ -7064,7 +7162,7 @@
     </row>
     <row r="70" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="21" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C70" s="22">
         <v>232.23</v>
@@ -7084,7 +7182,7 @@
     </row>
     <row r="71" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="18" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C71" s="19">
         <v>226.19</v>
@@ -7104,7 +7202,7 @@
     </row>
     <row r="72" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C72" s="22">
         <v>229.57</v>
@@ -7124,7 +7222,7 @@
     </row>
     <row r="73" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="18" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C73" s="19">
         <v>229.73</v>
@@ -7144,7 +7242,7 @@
     </row>
     <row r="74" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="21" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C74" s="22">
         <v>230.72</v>
@@ -7164,7 +7262,7 @@
     </row>
     <row r="75" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B75" s="18" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="C75" s="19">
         <v>227.06</v>
@@ -7184,7 +7282,7 @@
     </row>
     <row r="76" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B76" s="21" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C76" s="22">
         <v>228.15</v>
@@ -7204,7 +7302,7 @@
     </row>
     <row r="77" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B77" s="18" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C77" s="19">
         <v>232.16</v>
@@ -7224,7 +7322,7 @@
     </row>
     <row r="78" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B78" s="21" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C78" s="22">
         <v>235.65</v>
@@ -7244,7 +7342,7 @@
     </row>
     <row r="79" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B79" s="18" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C79" s="19">
         <v>234.86</v>
@@ -7264,7 +7362,7 @@
     </row>
     <row r="80" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B80" s="21" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C80" s="22">
         <v>234.65</v>
@@ -7284,7 +7382,7 @@
     </row>
     <row r="81" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B81" s="18" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="C81" s="19">
         <v>236.51</v>
@@ -7304,7 +7402,7 @@
     </row>
     <row r="82" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B82" s="21" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="C82" s="22">
         <v>232.62</v>
@@ -7324,7 +7422,7 @@
     </row>
     <row r="83" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B83" s="18" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C83" s="19">
         <v>232.8</v>
@@ -7344,7 +7442,7 @@
     </row>
     <row r="84" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B84" s="21" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C84" s="22">
         <v>233.03</v>
@@ -7364,7 +7462,7 @@
     </row>
     <row r="85" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B85" s="18" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C85" s="19">
         <v>233.69</v>
@@ -7384,7 +7482,7 @@
     </row>
     <row r="86" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B86" s="21" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C86" s="22">
         <v>235.58</v>
@@ -7404,7 +7502,7 @@
     </row>
     <row r="87" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B87" s="18" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C87" s="19">
         <v>235.85</v>
@@ -7424,7 +7522,7 @@
     </row>
     <row r="88" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B88" s="21" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C88" s="22">
         <v>235.15</v>
@@ -7444,7 +7542,7 @@
     </row>
     <row r="89" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B89" s="18" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C89" s="19">
         <v>232.81</v>
@@ -7464,7 +7562,7 @@
     </row>
     <row r="90" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B90" s="21" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C90" s="22">
         <v>234.55</v>
@@ -7484,7 +7582,7 @@
     </row>
     <row r="91" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B91" s="18" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C91" s="19">
         <v>235.65</v>
@@ -7504,7 +7602,7 @@
     </row>
     <row r="92" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B92" s="21" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C92" s="22">
         <v>232.85</v>
@@ -7524,7 +7622,7 @@
     </row>
     <row r="93" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B93" s="18" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C93" s="19">
         <v>233.46</v>
@@ -7544,7 +7642,7 @@
     </row>
     <row r="94" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B94" s="21" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C94" s="22">
         <v>235.49</v>
@@ -7564,7 +7662,7 @@
     </row>
     <row r="95" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B95" s="18" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C95" s="19">
         <v>233.68</v>
@@ -7584,7 +7682,7 @@
     </row>
     <row r="96" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B96" s="21" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C96" s="22">
         <v>230.18</v>
@@ -7604,7 +7702,7 @@
     </row>
     <row r="97" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B97" s="18" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C97" s="19">
         <v>227.59</v>
@@ -7624,7 +7722,7 @@
     </row>
     <row r="98" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B98" s="21" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C98" s="22">
         <v>230.76</v>
@@ -7644,7 +7742,7 @@
     </row>
     <row r="99" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B99" s="18" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C99" s="19">
         <v>234.41</v>
@@ -7664,7 +7762,7 @@
     </row>
     <row r="100" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B100" s="21" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C100" s="22">
         <v>236.33</v>
@@ -7684,7 +7782,7 @@
     </row>
     <row r="101" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B101" s="18" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C101" s="19">
         <v>236.59</v>
@@ -7704,7 +7802,7 @@
     </row>
     <row r="102" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B102" s="21" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C102" s="22">
         <v>233.27</v>
@@ -7724,7 +7822,7 @@
     </row>
     <row r="103" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B103" s="18" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C103" s="19">
         <v>235.85</v>
@@ -7744,7 +7842,7 @@
     </row>
     <row r="104" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B104" s="21" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C104" s="22">
         <v>234.74</v>
@@ -7764,7 +7862,7 @@
     </row>
     <row r="105" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B105" s="18" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C105" s="19">
         <v>230.69</v>
@@ -7784,7 +7882,7 @@
     </row>
     <row r="106" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B106" s="21" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C106" s="22">
         <v>230.74</v>
@@ -7804,7 +7902,7 @@
     </row>
     <row r="107" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B107" s="18" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C107" s="19">
         <v>233.7</v>
@@ -7824,7 +7922,7 @@
     </row>
     <row r="108" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B108" s="21" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C108" s="22">
         <v>233.91</v>
@@ -7844,7 +7942,7 @@
     </row>
     <row r="109" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B109" s="18" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C109" s="19">
         <v>235.18</v>
@@ -7864,7 +7962,7 @@
     </row>
     <row r="110" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B110" s="21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C110" s="22">
         <v>235.77</v>
@@ -7884,7 +7982,7 @@
     </row>
     <row r="111" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B111" s="18" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C111" s="19">
         <v>231.41</v>
@@ -7904,7 +8002,7 @@
     </row>
     <row r="112" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B112" s="21" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C112" s="22">
         <v>234.09</v>
@@ -7924,7 +8022,7 @@
     </row>
     <row r="113" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B113" s="18" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C113" s="19">
         <v>231.72</v>
@@ -7944,7 +8042,7 @@
     </row>
     <row r="114" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B114" s="21" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C114" s="22">
         <v>234.7</v>
@@ -7964,7 +8062,7 @@
     </row>
     <row r="115" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B115" s="18" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C115" s="19">
         <v>229.37</v>
@@ -7984,7 +8082,7 @@
     </row>
     <row r="116" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B116" s="21" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C116" s="22">
         <v>232.64</v>
@@ -8004,7 +8102,7 @@
     </row>
     <row r="117" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B117" s="18" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C117" s="19">
         <v>235.04</v>
@@ -8024,7 +8122,7 @@
     </row>
     <row r="118" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B118" s="21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C118" s="22">
         <v>235.39</v>
@@ -8044,7 +8142,7 @@
     </row>
     <row r="119" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B119" s="18" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C119" s="19">
         <v>233.2</v>
@@ -8064,7 +8162,7 @@
     </row>
     <row r="120" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B120" s="21" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C120" s="22">
         <v>232.66</v>
@@ -8084,7 +8182,7 @@
     </row>
     <row r="121" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B121" s="18" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C121" s="19">
         <v>228.54</v>
@@ -8104,7 +8202,7 @@
     </row>
     <row r="122" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B122" s="21" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C122" s="22">
         <v>227.22</v>
@@ -8124,7 +8222,7 @@
     </row>
     <row r="123" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B123" s="18" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C123" s="19">
         <v>232.76</v>
@@ -8144,7 +8242,7 @@
     </row>
     <row r="124" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B124" s="21" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C124" s="22">
         <v>231.4</v>
@@ -8164,7 +8262,7 @@
     </row>
     <row r="125" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B125" s="18" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="C125" s="19">
         <v>229.97</v>
@@ -8184,7 +8282,7 @@
     </row>
     <row r="126" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B126" s="21" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C126" s="22">
         <v>230.76</v>
@@ -8204,7 +8302,7 @@
     </row>
     <row r="127" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B127" s="18" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C127" s="19">
         <v>235.44</v>
@@ -8224,7 +8322,7 @@
     </row>
     <row r="128" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B128" s="21" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C128" s="22">
         <v>237.49</v>
@@ -8244,7 +8342,7 @@
     </row>
     <row r="129" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B129" s="18" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C129" s="19">
         <v>233.84</v>
@@ -8264,7 +8362,7 @@
     </row>
     <row r="130" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B130" s="21" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C130" s="22">
         <v>233.2</v>
@@ -8284,7 +8382,7 @@
     </row>
     <row r="131" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B131" s="18" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C131" s="19">
         <v>233.17</v>
@@ -8304,7 +8402,7 @@
     </row>
     <row r="132" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B132" s="21" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C132" s="22">
         <v>233.44</v>
@@ -8324,7 +8422,7 @@
     </row>
     <row r="133" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B133" s="18" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C133" s="19">
         <v>232.53</v>
@@ -8344,7 +8442,7 @@
     </row>
     <row r="134" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B134" s="21" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C134" s="22">
         <v>235.48</v>
@@ -8364,7 +8462,7 @@
     </row>
     <row r="135" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B135" s="18" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C135" s="19">
         <v>237.01</v>
@@ -8384,7 +8482,7 @@
     </row>
     <row r="136" spans="2:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B136" s="21" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C136" s="22">
         <v>240.73</v>
@@ -8430,54 +8528,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="81" t="s">
-        <v>280</v>
-      </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
+      <c r="B1" s="86" t="s">
+        <v>281</v>
+      </c>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
     </row>
     <row r="2" spans="2:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="94" t="s">
-        <v>281</v>
-      </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
+      <c r="B2" s="99" t="s">
+        <v>282</v>
+      </c>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
     </row>
     <row r="3" spans="2:9" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:9" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8488,22 +8586,22 @@
         <v>143</v>
       </c>
       <c r="D5" s="24" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G5" s="24" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H5" s="24" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="6" spans="2:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -8516,7 +8614,7 @@
         <v>199.69</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E6" s="22" t="str">
         <f>IF(ROW()-5&lt;7,"",AVERAGE(c0:C6))</f>
@@ -12908,473 +13006,473 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:32" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="78" t="s">
-        <v>297</v>
-      </c>
-      <c r="C1" s="68"/>
-      <c r="D1" s="68"/>
-      <c r="E1" s="68"/>
-      <c r="F1" s="68"/>
-      <c r="G1" s="68"/>
-      <c r="H1" s="68"/>
-      <c r="I1" s="68"/>
-      <c r="J1" s="68"/>
-      <c r="K1" s="68"/>
-      <c r="L1" s="68"/>
-      <c r="M1" s="68"/>
-      <c r="N1" s="68"/>
-      <c r="O1" s="68"/>
-      <c r="P1" s="68"/>
-      <c r="Q1" s="68"/>
-      <c r="R1" s="68"/>
-      <c r="S1" s="68"/>
-      <c r="T1" s="68"/>
-      <c r="U1" s="68"/>
-      <c r="V1" s="68"/>
-      <c r="W1" s="68"/>
-      <c r="X1" s="68"/>
-      <c r="Y1" s="68"/>
-      <c r="Z1" s="68"/>
-      <c r="AA1" s="68"/>
-      <c r="AB1" s="68"/>
-      <c r="AC1" s="68"/>
-      <c r="AD1" s="68"/>
-      <c r="AE1" s="68"/>
-      <c r="AF1" s="68"/>
+      <c r="B1" s="83" t="s">
+        <v>298</v>
+      </c>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
+      <c r="J1" s="73"/>
+      <c r="K1" s="73"/>
+      <c r="L1" s="73"/>
+      <c r="M1" s="73"/>
+      <c r="N1" s="73"/>
+      <c r="O1" s="73"/>
+      <c r="P1" s="73"/>
+      <c r="Q1" s="73"/>
+      <c r="R1" s="73"/>
+      <c r="S1" s="73"/>
+      <c r="T1" s="73"/>
+      <c r="U1" s="73"/>
+      <c r="V1" s="73"/>
+      <c r="W1" s="73"/>
+      <c r="X1" s="73"/>
+      <c r="Y1" s="73"/>
+      <c r="Z1" s="73"/>
+      <c r="AA1" s="73"/>
+      <c r="AB1" s="73"/>
+      <c r="AC1" s="73"/>
+      <c r="AD1" s="73"/>
+      <c r="AE1" s="73"/>
+      <c r="AF1" s="73"/>
     </row>
     <row r="2" spans="2:32" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="106" t="s">
-        <v>298</v>
-      </c>
-      <c r="C2" s="68"/>
-      <c r="D2" s="68"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="68"/>
-      <c r="G2" s="68"/>
-      <c r="H2" s="68"/>
-      <c r="I2" s="68"/>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="68"/>
-      <c r="N2" s="68"/>
-      <c r="O2" s="68"/>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="68"/>
-      <c r="R2" s="68"/>
-      <c r="S2" s="68"/>
-      <c r="T2" s="68"/>
-      <c r="U2" s="68"/>
-      <c r="V2" s="68"/>
-      <c r="W2" s="68"/>
-      <c r="X2" s="68"/>
-      <c r="Y2" s="68"/>
-      <c r="Z2" s="68"/>
-      <c r="AA2" s="68"/>
-      <c r="AB2" s="68"/>
-      <c r="AC2" s="68"/>
-      <c r="AD2" s="68"/>
-      <c r="AE2" s="68"/>
-      <c r="AF2" s="68"/>
+      <c r="B2" s="111" t="s">
+        <v>299</v>
+      </c>
+      <c r="C2" s="73"/>
+      <c r="D2" s="73"/>
+      <c r="E2" s="73"/>
+      <c r="F2" s="73"/>
+      <c r="G2" s="73"/>
+      <c r="H2" s="73"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="73"/>
+      <c r="L2" s="73"/>
+      <c r="M2" s="73"/>
+      <c r="N2" s="73"/>
+      <c r="O2" s="73"/>
+      <c r="P2" s="73"/>
+      <c r="Q2" s="73"/>
+      <c r="R2" s="73"/>
+      <c r="S2" s="73"/>
+      <c r="T2" s="73"/>
+      <c r="U2" s="73"/>
+      <c r="V2" s="73"/>
+      <c r="W2" s="73"/>
+      <c r="X2" s="73"/>
+      <c r="Y2" s="73"/>
+      <c r="Z2" s="73"/>
+      <c r="AA2" s="73"/>
+      <c r="AB2" s="73"/>
+      <c r="AC2" s="73"/>
+      <c r="AD2" s="73"/>
+      <c r="AE2" s="73"/>
+      <c r="AF2" s="73"/>
     </row>
     <row r="3" spans="2:32" ht="7.5" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:32" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="102" t="s">
-        <v>299</v>
-      </c>
-      <c r="C4" s="68"/>
-      <c r="D4" s="68"/>
-      <c r="E4" s="68"/>
-      <c r="F4" s="68"/>
-      <c r="G4" s="68"/>
-      <c r="H4" s="68"/>
-      <c r="I4" s="99" t="s">
+      <c r="B4" s="107" t="s">
         <v>300</v>
       </c>
-      <c r="J4" s="68"/>
-      <c r="K4" s="68"/>
-      <c r="L4" s="68"/>
-      <c r="M4" s="68"/>
-      <c r="N4" s="68"/>
-      <c r="O4" s="68"/>
-      <c r="P4" s="103" t="s">
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
+      <c r="H4" s="73"/>
+      <c r="I4" s="104" t="s">
         <v>301</v>
       </c>
-      <c r="Q4" s="68"/>
-      <c r="R4" s="68"/>
-      <c r="S4" s="68"/>
-      <c r="T4" s="68"/>
-      <c r="U4" s="68"/>
-      <c r="V4" s="68"/>
-      <c r="W4" s="101" t="s">
+      <c r="J4" s="73"/>
+      <c r="K4" s="73"/>
+      <c r="L4" s="73"/>
+      <c r="M4" s="73"/>
+      <c r="N4" s="73"/>
+      <c r="O4" s="73"/>
+      <c r="P4" s="108" t="s">
         <v>302</v>
       </c>
-      <c r="X4" s="68"/>
-      <c r="Y4" s="68"/>
-      <c r="Z4" s="68"/>
-      <c r="AA4" s="68"/>
-      <c r="AB4" s="68"/>
-      <c r="AC4" s="68"/>
+      <c r="Q4" s="73"/>
+      <c r="R4" s="73"/>
+      <c r="S4" s="73"/>
+      <c r="T4" s="73"/>
+      <c r="U4" s="73"/>
+      <c r="V4" s="73"/>
+      <c r="W4" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="X4" s="73"/>
+      <c r="Y4" s="73"/>
+      <c r="Z4" s="73"/>
+      <c r="AA4" s="73"/>
+      <c r="AB4" s="73"/>
+      <c r="AC4" s="73"/>
     </row>
     <row r="5" spans="2:32" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="105">
+      <c r="B5" s="110">
         <f>'📊 RAW DATA'!F7</f>
         <v>199.69</v>
       </c>
-      <c r="C5" s="68"/>
-      <c r="D5" s="68"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="68"/>
-      <c r="G5" s="68"/>
-      <c r="H5" s="68"/>
-      <c r="I5" s="104">
+      <c r="C5" s="73"/>
+      <c r="D5" s="73"/>
+      <c r="E5" s="73"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="109">
         <f>'📊 RAW DATA'!F136</f>
         <v>238.77</v>
       </c>
-      <c r="J5" s="68"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="68"/>
-      <c r="N5" s="68"/>
-      <c r="O5" s="68"/>
-      <c r="P5" s="107">
+      <c r="J5" s="73"/>
+      <c r="K5" s="73"/>
+      <c r="L5" s="73"/>
+      <c r="M5" s="73"/>
+      <c r="N5" s="73"/>
+      <c r="O5" s="73"/>
+      <c r="P5" s="112">
         <f>('📊 RAW DATA'!F136-'📊 RAW DATA'!F7)/'📊 RAW DATA'!F7</f>
         <v>0.19570334017727484</v>
       </c>
-      <c r="Q5" s="68"/>
-      <c r="R5" s="68"/>
-      <c r="S5" s="68"/>
-      <c r="T5" s="68"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="98" t="str">
+      <c r="Q5" s="73"/>
+      <c r="R5" s="73"/>
+      <c r="S5" s="73"/>
+      <c r="T5" s="73"/>
+      <c r="U5" s="73"/>
+      <c r="V5" s="73"/>
+      <c r="W5" s="103" t="str">
         <f>'🔬 ANALYSIS'!H135</f>
         <v>BUY ▲</v>
       </c>
-      <c r="X5" s="68"/>
-      <c r="Y5" s="68"/>
-      <c r="Z5" s="68"/>
-      <c r="AA5" s="68"/>
-      <c r="AB5" s="68"/>
-      <c r="AC5" s="68"/>
+      <c r="X5" s="73"/>
+      <c r="Y5" s="73"/>
+      <c r="Z5" s="73"/>
+      <c r="AA5" s="73"/>
+      <c r="AB5" s="73"/>
+      <c r="AC5" s="73"/>
     </row>
     <row r="6" spans="2:32" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="68"/>
-      <c r="C6" s="68"/>
-      <c r="D6" s="68"/>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="68"/>
-      <c r="J6" s="68"/>
-      <c r="K6" s="68"/>
-      <c r="L6" s="68"/>
-      <c r="M6" s="68"/>
-      <c r="N6" s="68"/>
-      <c r="O6" s="68"/>
-      <c r="P6" s="68"/>
-      <c r="Q6" s="68"/>
-      <c r="R6" s="68"/>
-      <c r="S6" s="68"/>
-      <c r="T6" s="68"/>
-      <c r="U6" s="68"/>
-      <c r="V6" s="68"/>
-      <c r="W6" s="68"/>
-      <c r="X6" s="68"/>
-      <c r="Y6" s="68"/>
-      <c r="Z6" s="68"/>
-      <c r="AA6" s="68"/>
-      <c r="AB6" s="68"/>
-      <c r="AC6" s="68"/>
+      <c r="B6" s="73"/>
+      <c r="C6" s="73"/>
+      <c r="D6" s="73"/>
+      <c r="E6" s="73"/>
+      <c r="F6" s="73"/>
+      <c r="G6" s="73"/>
+      <c r="H6" s="73"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="73"/>
+      <c r="L6" s="73"/>
+      <c r="M6" s="73"/>
+      <c r="N6" s="73"/>
+      <c r="O6" s="73"/>
+      <c r="P6" s="73"/>
+      <c r="Q6" s="73"/>
+      <c r="R6" s="73"/>
+      <c r="S6" s="73"/>
+      <c r="T6" s="73"/>
+      <c r="U6" s="73"/>
+      <c r="V6" s="73"/>
+      <c r="W6" s="73"/>
+      <c r="X6" s="73"/>
+      <c r="Y6" s="73"/>
+      <c r="Z6" s="73"/>
+      <c r="AA6" s="73"/>
+      <c r="AB6" s="73"/>
+      <c r="AC6" s="73"/>
     </row>
     <row r="7" spans="2:32" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="91"/>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
-      <c r="F7" s="68"/>
-      <c r="G7" s="68"/>
-      <c r="H7" s="68"/>
-      <c r="I7" s="83"/>
-      <c r="J7" s="68"/>
-      <c r="K7" s="68"/>
-      <c r="L7" s="68"/>
-      <c r="M7" s="68"/>
-      <c r="N7" s="68"/>
-      <c r="O7" s="68"/>
-      <c r="P7" s="82"/>
-      <c r="Q7" s="68"/>
-      <c r="R7" s="68"/>
-      <c r="S7" s="68"/>
-      <c r="T7" s="68"/>
-      <c r="U7" s="68"/>
-      <c r="V7" s="68"/>
-      <c r="W7" s="108"/>
-      <c r="X7" s="68"/>
-      <c r="Y7" s="68"/>
-      <c r="Z7" s="68"/>
-      <c r="AA7" s="68"/>
-      <c r="AB7" s="68"/>
-      <c r="AC7" s="68"/>
+      <c r="B7" s="95"/>
+      <c r="C7" s="73"/>
+      <c r="D7" s="73"/>
+      <c r="E7" s="73"/>
+      <c r="F7" s="73"/>
+      <c r="G7" s="73"/>
+      <c r="H7" s="73"/>
+      <c r="I7" s="88"/>
+      <c r="J7" s="73"/>
+      <c r="K7" s="73"/>
+      <c r="L7" s="73"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="73"/>
+      <c r="P7" s="87"/>
+      <c r="Q7" s="73"/>
+      <c r="R7" s="73"/>
+      <c r="S7" s="73"/>
+      <c r="T7" s="73"/>
+      <c r="U7" s="73"/>
+      <c r="V7" s="73"/>
+      <c r="W7" s="113"/>
+      <c r="X7" s="73"/>
+      <c r="Y7" s="73"/>
+      <c r="Z7" s="73"/>
+      <c r="AA7" s="73"/>
+      <c r="AB7" s="73"/>
+      <c r="AC7" s="73"/>
     </row>
     <row r="8" spans="2:32" ht="6" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="34" spans="2:32" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="96" t="s">
-        <v>303</v>
-      </c>
-      <c r="C34" s="68"/>
-      <c r="D34" s="68"/>
-      <c r="E34" s="68"/>
-      <c r="F34" s="68"/>
-      <c r="G34" s="68"/>
-      <c r="H34" s="68"/>
-      <c r="I34" s="68"/>
-      <c r="J34" s="68"/>
-      <c r="K34" s="68"/>
-      <c r="L34" s="68"/>
-      <c r="M34" s="68"/>
-      <c r="N34" s="68"/>
-      <c r="O34" s="68"/>
-      <c r="P34" s="68"/>
-      <c r="Q34" s="68"/>
-      <c r="R34" s="68"/>
-      <c r="S34" s="68"/>
-      <c r="T34" s="68"/>
-      <c r="U34" s="68"/>
-      <c r="V34" s="68"/>
-      <c r="W34" s="68"/>
-      <c r="X34" s="68"/>
-      <c r="Y34" s="68"/>
-      <c r="Z34" s="68"/>
-      <c r="AA34" s="68"/>
-      <c r="AB34" s="68"/>
-      <c r="AC34" s="68"/>
-      <c r="AD34" s="68"/>
-      <c r="AE34" s="68"/>
-      <c r="AF34" s="68"/>
+      <c r="B34" s="101" t="s">
+        <v>304</v>
+      </c>
+      <c r="C34" s="73"/>
+      <c r="D34" s="73"/>
+      <c r="E34" s="73"/>
+      <c r="F34" s="73"/>
+      <c r="G34" s="73"/>
+      <c r="H34" s="73"/>
+      <c r="I34" s="73"/>
+      <c r="J34" s="73"/>
+      <c r="K34" s="73"/>
+      <c r="L34" s="73"/>
+      <c r="M34" s="73"/>
+      <c r="N34" s="73"/>
+      <c r="O34" s="73"/>
+      <c r="P34" s="73"/>
+      <c r="Q34" s="73"/>
+      <c r="R34" s="73"/>
+      <c r="S34" s="73"/>
+      <c r="T34" s="73"/>
+      <c r="U34" s="73"/>
+      <c r="V34" s="73"/>
+      <c r="W34" s="73"/>
+      <c r="X34" s="73"/>
+      <c r="Y34" s="73"/>
+      <c r="Z34" s="73"/>
+      <c r="AA34" s="73"/>
+      <c r="AB34" s="73"/>
+      <c r="AC34" s="73"/>
+      <c r="AD34" s="73"/>
+      <c r="AE34" s="73"/>
+      <c r="AF34" s="73"/>
     </row>
     <row r="35" spans="2:32" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="97" t="s">
-        <v>304</v>
-      </c>
-      <c r="C35" s="68"/>
-      <c r="D35" s="68"/>
-      <c r="E35" s="68"/>
-      <c r="F35" s="68"/>
-      <c r="G35" s="68"/>
-      <c r="H35" s="68"/>
-      <c r="I35" s="68"/>
-      <c r="J35" s="68"/>
-      <c r="K35" s="68"/>
-      <c r="L35" s="100" t="s">
+      <c r="B35" s="102" t="s">
         <v>305</v>
       </c>
-      <c r="M35" s="68"/>
-      <c r="N35" s="68"/>
-      <c r="O35" s="68"/>
-      <c r="P35" s="68"/>
-      <c r="Q35" s="68"/>
-      <c r="R35" s="68"/>
-      <c r="S35" s="68"/>
-      <c r="T35" s="68"/>
-      <c r="U35" s="68"/>
-      <c r="V35" s="68"/>
-      <c r="W35" s="68"/>
-      <c r="X35" s="68"/>
-      <c r="Y35" s="68"/>
-      <c r="Z35" s="68"/>
-      <c r="AA35" s="68"/>
-      <c r="AB35" s="68"/>
-      <c r="AC35" s="68"/>
-      <c r="AD35" s="68"/>
-      <c r="AE35" s="68"/>
-      <c r="AF35" s="68"/>
+      <c r="C35" s="73"/>
+      <c r="D35" s="73"/>
+      <c r="E35" s="73"/>
+      <c r="F35" s="73"/>
+      <c r="G35" s="73"/>
+      <c r="H35" s="73"/>
+      <c r="I35" s="73"/>
+      <c r="J35" s="73"/>
+      <c r="K35" s="73"/>
+      <c r="L35" s="105" t="s">
+        <v>306</v>
+      </c>
+      <c r="M35" s="73"/>
+      <c r="N35" s="73"/>
+      <c r="O35" s="73"/>
+      <c r="P35" s="73"/>
+      <c r="Q35" s="73"/>
+      <c r="R35" s="73"/>
+      <c r="S35" s="73"/>
+      <c r="T35" s="73"/>
+      <c r="U35" s="73"/>
+      <c r="V35" s="73"/>
+      <c r="W35" s="73"/>
+      <c r="X35" s="73"/>
+      <c r="Y35" s="73"/>
+      <c r="Z35" s="73"/>
+      <c r="AA35" s="73"/>
+      <c r="AB35" s="73"/>
+      <c r="AC35" s="73"/>
+      <c r="AD35" s="73"/>
+      <c r="AE35" s="73"/>
+      <c r="AF35" s="73"/>
     </row>
     <row r="36" spans="2:32" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="97" t="s">
-        <v>306</v>
-      </c>
-      <c r="C36" s="68"/>
-      <c r="D36" s="68"/>
-      <c r="E36" s="68"/>
-      <c r="F36" s="68"/>
-      <c r="G36" s="68"/>
-      <c r="H36" s="68"/>
-      <c r="I36" s="68"/>
-      <c r="J36" s="68"/>
-      <c r="K36" s="68"/>
-      <c r="L36" s="100" t="s">
+      <c r="B36" s="102" t="s">
         <v>307</v>
       </c>
-      <c r="M36" s="68"/>
-      <c r="N36" s="68"/>
-      <c r="O36" s="68"/>
-      <c r="P36" s="68"/>
-      <c r="Q36" s="68"/>
-      <c r="R36" s="68"/>
-      <c r="S36" s="68"/>
-      <c r="T36" s="68"/>
-      <c r="U36" s="68"/>
-      <c r="V36" s="68"/>
-      <c r="W36" s="68"/>
-      <c r="X36" s="68"/>
-      <c r="Y36" s="68"/>
-      <c r="Z36" s="68"/>
-      <c r="AA36" s="68"/>
-      <c r="AB36" s="68"/>
-      <c r="AC36" s="68"/>
-      <c r="AD36" s="68"/>
-      <c r="AE36" s="68"/>
-      <c r="AF36" s="68"/>
+      <c r="C36" s="73"/>
+      <c r="D36" s="73"/>
+      <c r="E36" s="73"/>
+      <c r="F36" s="73"/>
+      <c r="G36" s="73"/>
+      <c r="H36" s="73"/>
+      <c r="I36" s="73"/>
+      <c r="J36" s="73"/>
+      <c r="K36" s="73"/>
+      <c r="L36" s="105" t="s">
+        <v>308</v>
+      </c>
+      <c r="M36" s="73"/>
+      <c r="N36" s="73"/>
+      <c r="O36" s="73"/>
+      <c r="P36" s="73"/>
+      <c r="Q36" s="73"/>
+      <c r="R36" s="73"/>
+      <c r="S36" s="73"/>
+      <c r="T36" s="73"/>
+      <c r="U36" s="73"/>
+      <c r="V36" s="73"/>
+      <c r="W36" s="73"/>
+      <c r="X36" s="73"/>
+      <c r="Y36" s="73"/>
+      <c r="Z36" s="73"/>
+      <c r="AA36" s="73"/>
+      <c r="AB36" s="73"/>
+      <c r="AC36" s="73"/>
+      <c r="AD36" s="73"/>
+      <c r="AE36" s="73"/>
+      <c r="AF36" s="73"/>
     </row>
     <row r="37" spans="2:32" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="97" t="s">
-        <v>308</v>
-      </c>
-      <c r="C37" s="68"/>
-      <c r="D37" s="68"/>
-      <c r="E37" s="68"/>
-      <c r="F37" s="68"/>
-      <c r="G37" s="68"/>
-      <c r="H37" s="68"/>
-      <c r="I37" s="68"/>
-      <c r="J37" s="68"/>
-      <c r="K37" s="68"/>
-      <c r="L37" s="100" t="s">
+      <c r="B37" s="102" t="s">
         <v>309</v>
       </c>
-      <c r="M37" s="68"/>
-      <c r="N37" s="68"/>
-      <c r="O37" s="68"/>
-      <c r="P37" s="68"/>
-      <c r="Q37" s="68"/>
-      <c r="R37" s="68"/>
-      <c r="S37" s="68"/>
-      <c r="T37" s="68"/>
-      <c r="U37" s="68"/>
-      <c r="V37" s="68"/>
-      <c r="W37" s="68"/>
-      <c r="X37" s="68"/>
-      <c r="Y37" s="68"/>
-      <c r="Z37" s="68"/>
-      <c r="AA37" s="68"/>
-      <c r="AB37" s="68"/>
-      <c r="AC37" s="68"/>
-      <c r="AD37" s="68"/>
-      <c r="AE37" s="68"/>
-      <c r="AF37" s="68"/>
+      <c r="C37" s="73"/>
+      <c r="D37" s="73"/>
+      <c r="E37" s="73"/>
+      <c r="F37" s="73"/>
+      <c r="G37" s="73"/>
+      <c r="H37" s="73"/>
+      <c r="I37" s="73"/>
+      <c r="J37" s="73"/>
+      <c r="K37" s="73"/>
+      <c r="L37" s="105" t="s">
+        <v>310</v>
+      </c>
+      <c r="M37" s="73"/>
+      <c r="N37" s="73"/>
+      <c r="O37" s="73"/>
+      <c r="P37" s="73"/>
+      <c r="Q37" s="73"/>
+      <c r="R37" s="73"/>
+      <c r="S37" s="73"/>
+      <c r="T37" s="73"/>
+      <c r="U37" s="73"/>
+      <c r="V37" s="73"/>
+      <c r="W37" s="73"/>
+      <c r="X37" s="73"/>
+      <c r="Y37" s="73"/>
+      <c r="Z37" s="73"/>
+      <c r="AA37" s="73"/>
+      <c r="AB37" s="73"/>
+      <c r="AC37" s="73"/>
+      <c r="AD37" s="73"/>
+      <c r="AE37" s="73"/>
+      <c r="AF37" s="73"/>
     </row>
     <row r="38" spans="2:32" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="97" t="s">
-        <v>310</v>
-      </c>
-      <c r="C38" s="68"/>
-      <c r="D38" s="68"/>
-      <c r="E38" s="68"/>
-      <c r="F38" s="68"/>
-      <c r="G38" s="68"/>
-      <c r="H38" s="68"/>
-      <c r="I38" s="68"/>
-      <c r="J38" s="68"/>
-      <c r="K38" s="68"/>
-      <c r="L38" s="100" t="s">
+      <c r="B38" s="102" t="s">
         <v>311</v>
       </c>
-      <c r="M38" s="68"/>
-      <c r="N38" s="68"/>
-      <c r="O38" s="68"/>
-      <c r="P38" s="68"/>
-      <c r="Q38" s="68"/>
-      <c r="R38" s="68"/>
-      <c r="S38" s="68"/>
-      <c r="T38" s="68"/>
-      <c r="U38" s="68"/>
-      <c r="V38" s="68"/>
-      <c r="W38" s="68"/>
-      <c r="X38" s="68"/>
-      <c r="Y38" s="68"/>
-      <c r="Z38" s="68"/>
-      <c r="AA38" s="68"/>
-      <c r="AB38" s="68"/>
-      <c r="AC38" s="68"/>
-      <c r="AD38" s="68"/>
-      <c r="AE38" s="68"/>
-      <c r="AF38" s="68"/>
+      <c r="C38" s="73"/>
+      <c r="D38" s="73"/>
+      <c r="E38" s="73"/>
+      <c r="F38" s="73"/>
+      <c r="G38" s="73"/>
+      <c r="H38" s="73"/>
+      <c r="I38" s="73"/>
+      <c r="J38" s="73"/>
+      <c r="K38" s="73"/>
+      <c r="L38" s="105" t="s">
+        <v>312</v>
+      </c>
+      <c r="M38" s="73"/>
+      <c r="N38" s="73"/>
+      <c r="O38" s="73"/>
+      <c r="P38" s="73"/>
+      <c r="Q38" s="73"/>
+      <c r="R38" s="73"/>
+      <c r="S38" s="73"/>
+      <c r="T38" s="73"/>
+      <c r="U38" s="73"/>
+      <c r="V38" s="73"/>
+      <c r="W38" s="73"/>
+      <c r="X38" s="73"/>
+      <c r="Y38" s="73"/>
+      <c r="Z38" s="73"/>
+      <c r="AA38" s="73"/>
+      <c r="AB38" s="73"/>
+      <c r="AC38" s="73"/>
+      <c r="AD38" s="73"/>
+      <c r="AE38" s="73"/>
+      <c r="AF38" s="73"/>
     </row>
     <row r="39" spans="2:32" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="97" t="s">
-        <v>312</v>
-      </c>
-      <c r="C39" s="68"/>
-      <c r="D39" s="68"/>
-      <c r="E39" s="68"/>
-      <c r="F39" s="68"/>
-      <c r="G39" s="68"/>
-      <c r="H39" s="68"/>
-      <c r="I39" s="68"/>
-      <c r="J39" s="68"/>
-      <c r="K39" s="68"/>
-      <c r="L39" s="100" t="s">
+      <c r="B39" s="102" t="s">
         <v>313</v>
       </c>
-      <c r="M39" s="68"/>
-      <c r="N39" s="68"/>
-      <c r="O39" s="68"/>
-      <c r="P39" s="68"/>
-      <c r="Q39" s="68"/>
-      <c r="R39" s="68"/>
-      <c r="S39" s="68"/>
-      <c r="T39" s="68"/>
-      <c r="U39" s="68"/>
-      <c r="V39" s="68"/>
-      <c r="W39" s="68"/>
-      <c r="X39" s="68"/>
-      <c r="Y39" s="68"/>
-      <c r="Z39" s="68"/>
-      <c r="AA39" s="68"/>
-      <c r="AB39" s="68"/>
-      <c r="AC39" s="68"/>
-      <c r="AD39" s="68"/>
-      <c r="AE39" s="68"/>
-      <c r="AF39" s="68"/>
+      <c r="C39" s="73"/>
+      <c r="D39" s="73"/>
+      <c r="E39" s="73"/>
+      <c r="F39" s="73"/>
+      <c r="G39" s="73"/>
+      <c r="H39" s="73"/>
+      <c r="I39" s="73"/>
+      <c r="J39" s="73"/>
+      <c r="K39" s="73"/>
+      <c r="L39" s="105" t="s">
+        <v>314</v>
+      </c>
+      <c r="M39" s="73"/>
+      <c r="N39" s="73"/>
+      <c r="O39" s="73"/>
+      <c r="P39" s="73"/>
+      <c r="Q39" s="73"/>
+      <c r="R39" s="73"/>
+      <c r="S39" s="73"/>
+      <c r="T39" s="73"/>
+      <c r="U39" s="73"/>
+      <c r="V39" s="73"/>
+      <c r="W39" s="73"/>
+      <c r="X39" s="73"/>
+      <c r="Y39" s="73"/>
+      <c r="Z39" s="73"/>
+      <c r="AA39" s="73"/>
+      <c r="AB39" s="73"/>
+      <c r="AC39" s="73"/>
+      <c r="AD39" s="73"/>
+      <c r="AE39" s="73"/>
+      <c r="AF39" s="73"/>
     </row>
     <row r="40" spans="2:32" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="97" t="s">
-        <v>314</v>
-      </c>
-      <c r="C40" s="68"/>
-      <c r="D40" s="68"/>
-      <c r="E40" s="68"/>
-      <c r="F40" s="68"/>
-      <c r="G40" s="68"/>
-      <c r="H40" s="68"/>
-      <c r="I40" s="68"/>
-      <c r="J40" s="68"/>
-      <c r="K40" s="68"/>
-      <c r="L40" s="100" t="s">
+      <c r="B40" s="102" t="s">
         <v>315</v>
       </c>
-      <c r="M40" s="68"/>
-      <c r="N40" s="68"/>
-      <c r="O40" s="68"/>
-      <c r="P40" s="68"/>
-      <c r="Q40" s="68"/>
-      <c r="R40" s="68"/>
-      <c r="S40" s="68"/>
-      <c r="T40" s="68"/>
-      <c r="U40" s="68"/>
-      <c r="V40" s="68"/>
-      <c r="W40" s="68"/>
-      <c r="X40" s="68"/>
-      <c r="Y40" s="68"/>
-      <c r="Z40" s="68"/>
-      <c r="AA40" s="68"/>
-      <c r="AB40" s="68"/>
-      <c r="AC40" s="68"/>
-      <c r="AD40" s="68"/>
-      <c r="AE40" s="68"/>
-      <c r="AF40" s="68"/>
+      <c r="C40" s="73"/>
+      <c r="D40" s="73"/>
+      <c r="E40" s="73"/>
+      <c r="F40" s="73"/>
+      <c r="G40" s="73"/>
+      <c r="H40" s="73"/>
+      <c r="I40" s="73"/>
+      <c r="J40" s="73"/>
+      <c r="K40" s="73"/>
+      <c r="L40" s="105" t="s">
+        <v>316</v>
+      </c>
+      <c r="M40" s="73"/>
+      <c r="N40" s="73"/>
+      <c r="O40" s="73"/>
+      <c r="P40" s="73"/>
+      <c r="Q40" s="73"/>
+      <c r="R40" s="73"/>
+      <c r="S40" s="73"/>
+      <c r="T40" s="73"/>
+      <c r="U40" s="73"/>
+      <c r="V40" s="73"/>
+      <c r="W40" s="73"/>
+      <c r="X40" s="73"/>
+      <c r="Y40" s="73"/>
+      <c r="Z40" s="73"/>
+      <c r="AA40" s="73"/>
+      <c r="AB40" s="73"/>
+      <c r="AC40" s="73"/>
+      <c r="AD40" s="73"/>
+      <c r="AE40" s="73"/>
+      <c r="AF40" s="73"/>
     </row>
   </sheetData>
   <mergeCells count="27">
@@ -13383,7 +13481,7 @@
     <mergeCell ref="P7:V7"/>
     <mergeCell ref="L37:AF37"/>
     <mergeCell ref="B37:K37"/>
-    <mergeCell ref="B39:K39"/>
+    <mergeCell ref="I7:O7"/>
     <mergeCell ref="L36:AF36"/>
     <mergeCell ref="B5:H6"/>
     <mergeCell ref="B2:AF2"/>
@@ -13404,7 +13502,7 @@
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="L40:AF40"/>
     <mergeCell ref="I5:O6"/>
-    <mergeCell ref="I7:O7"/>
+    <mergeCell ref="B39:K39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>